<commit_message>
new dac model as th carrier
</commit_message>
<xml_diff>
--- a/data/SFI_ALD_Petrochemicals_Sample_EU_NA_Apr_2022.xlsx
+++ b/data/SFI_ALD_Petrochemicals_Sample_EU_NA_Apr_2022.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\plants_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D7989E9-420B-470D-942E-9C0588D68AF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -31256,15 +31256,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="c95907cf-e9f9-4b92-a10f-5d23f887974d">
@@ -31272,6 +31263,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -31293,14 +31293,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DF01CBF-A5C4-4282-859D-8EAB800F0387}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55D8B328-D93F-4E0D-94E2-653BFEE7AE74}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
@@ -31317,4 +31309,12 @@
     <ds:schemaRef ds:uri="c95907cf-e9f9-4b92-a10f-5d23f887974d"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DF01CBF-A5C4-4282-859D-8EAB800F0387}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
new investigation on base case study 2050
</commit_message>
<xml_diff>
--- a/data/SFI_ALD_Petrochemicals_Sample_EU_NA_Apr_2022.xlsx
+++ b/data/SFI_ALD_Petrochemicals_Sample_EU_NA_Apr_2022.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D7989E9-420B-470D-942E-9C0588D68AF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{311237B4-33E8-41AB-90D4-07D13ECA35B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-360" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{49FED9BB-E9B4-4298-B606-A2033C4439F2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{49FED9BB-E9B4-4298-B606-A2033C4439F2}"/>
   </bookViews>
   <sheets>
     <sheet name="About - General" sheetId="2" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5843" uniqueCount="1441">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5857" uniqueCount="1443">
   <si>
     <t>Spatial Finance Initiative Petrochemicals Database for Europe and North America (April 2022)</t>
   </si>
@@ -4489,6 +4489,12 @@
   </si>
   <si>
     <t>https://www.pbl.nl/en/publications/decarbonisation-options-for-large-volume-organic-chemicals-production-dow-terneuzen#:~:text=The%20most%20important%20facilities%20in,polyolefins%2C%20polyols%20and%20styrene%20rubbers.</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>https://www.icis.com/explore/resources/news/2023/01/18/10846094/insight-poor-demand-high-costs-stifle-europe-industry-despite-falling-gas-prices/</t>
   </si>
 </sst>
 </file>
@@ -5069,14 +5075,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9008B2CA-3D0D-4C83-BA51-A4822FB11F35}">
   <dimension ref="A1:D54"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.85546875" style="18" customWidth="1"/>
-    <col min="2" max="2" width="29.28515625" customWidth="1"/>
-    <col min="3" max="3" width="100.85546875" customWidth="1"/>
+    <col min="1" max="1" width="5.88671875" style="18" customWidth="1"/>
+    <col min="2" max="2" width="29.33203125" customWidth="1"/>
+    <col min="3" max="3" width="100.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="29"/>
       <c r="B1" s="32" t="s">
         <v>0</v>
@@ -5084,85 +5090,85 @@
       <c r="C1" s="32"/>
       <c r="D1" s="32"/>
     </row>
-    <row r="2" spans="1:4" ht="6.4" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:4" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="6.45" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:4" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="34" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="34"/>
       <c r="C3" s="34"/>
     </row>
-    <row r="4" spans="1:4" ht="9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ht="9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="15"/>
       <c r="B4" s="14"/>
       <c r="C4" s="14"/>
     </row>
-    <row r="5" spans="1:4" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="34" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="34"/>
       <c r="C5" s="34"/>
     </row>
-    <row r="6" spans="1:4" ht="9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ht="9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="15"/>
       <c r="B6" s="14"/>
       <c r="C6" s="14"/>
     </row>
-    <row r="7" spans="1:4" ht="47.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" ht="47.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="33" t="s">
         <v>3</v>
       </c>
       <c r="B7" s="33"/>
       <c r="C7" s="33"/>
     </row>
-    <row r="8" spans="1:4" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" ht="5.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="19"/>
       <c r="B8" s="19"/>
       <c r="C8" s="19"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="34" t="s">
         <v>1427</v>
       </c>
       <c r="B9" s="34"/>
       <c r="C9" s="34"/>
     </row>
-    <row r="10" spans="1:4" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" ht="9.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="19"/>
       <c r="B10" s="19"/>
       <c r="C10" s="19"/>
     </row>
-    <row r="11" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="33" t="s">
         <v>1426</v>
       </c>
       <c r="B11" s="33"/>
       <c r="C11" s="33"/>
     </row>
-    <row r="12" spans="1:4" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" ht="9.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="19"/>
       <c r="B12" s="19"/>
       <c r="C12" s="19"/>
     </row>
-    <row r="13" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="33" t="s">
         <v>4</v>
       </c>
       <c r="B13" s="33"/>
       <c r="C13" s="33"/>
     </row>
-    <row r="14" spans="1:4" ht="9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" ht="9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="15"/>
       <c r="B14" s="14"/>
       <c r="C14" s="14"/>
     </row>
-    <row r="15" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" s="16" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="17">
         <v>1</v>
       </c>
@@ -5173,7 +5179,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="17">
         <v>2</v>
       </c>
@@ -5184,7 +5190,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="17">
         <v>3</v>
       </c>
@@ -5195,7 +5201,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="17">
         <v>4</v>
       </c>
@@ -5206,7 +5212,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="17">
         <v>5</v>
       </c>
@@ -5217,7 +5223,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="17">
         <v>6</v>
       </c>
@@ -5228,7 +5234,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="17">
         <v>7</v>
       </c>
@@ -5239,7 +5245,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="17">
         <v>8</v>
       </c>
@@ -5250,7 +5256,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="17">
         <v>9</v>
       </c>
@@ -5261,7 +5267,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="17">
         <v>10</v>
       </c>
@@ -5272,7 +5278,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="17">
         <v>11</v>
       </c>
@@ -5283,7 +5289,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="17">
         <v>12</v>
       </c>
@@ -5294,7 +5300,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="17">
         <v>13</v>
       </c>
@@ -5305,7 +5311,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="17">
         <v>14</v>
       </c>
@@ -5316,7 +5322,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="17">
         <v>15</v>
       </c>
@@ -5327,7 +5333,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="17">
         <v>16</v>
       </c>
@@ -5338,7 +5344,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="17">
         <v>17</v>
       </c>
@@ -5349,7 +5355,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="17">
         <v>18</v>
       </c>
@@ -5360,7 +5366,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" s="17">
         <v>19</v>
       </c>
@@ -5371,7 +5377,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="17">
         <v>20</v>
       </c>
@@ -5382,7 +5388,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" s="17">
         <v>21</v>
       </c>
@@ -5393,7 +5399,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" s="17">
         <v>22</v>
       </c>
@@ -5404,7 +5410,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" s="17">
         <v>23</v>
       </c>
@@ -5415,7 +5421,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A40" s="17">
         <v>24</v>
       </c>
@@ -5426,7 +5432,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" s="17">
         <v>25</v>
       </c>
@@ -5437,7 +5443,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" s="17">
         <v>26</v>
       </c>
@@ -5448,7 +5454,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" s="17">
         <v>27</v>
       </c>
@@ -5459,7 +5465,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" s="17">
         <v>28</v>
       </c>
@@ -5470,7 +5476,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" s="17">
         <v>29</v>
       </c>
@@ -5481,7 +5487,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" s="17">
         <v>30</v>
       </c>
@@ -5492,7 +5498,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" s="17">
         <v>31</v>
       </c>
@@ -5503,7 +5509,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" s="17">
         <v>32</v>
       </c>
@@ -5514,7 +5520,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" s="17">
         <v>33</v>
       </c>
@@ -5525,7 +5531,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" s="17">
         <v>34</v>
       </c>
@@ -5536,7 +5542,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" s="17">
         <v>35</v>
       </c>
@@ -5547,14 +5553,14 @@
         <v>75</v>
       </c>
     </row>
-    <row r="53" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="34" t="s">
         <v>76</v>
       </c>
       <c r="B53" s="34"/>
       <c r="C53" s="34"/>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" s="18" t="s">
         <v>77</v>
       </c>
@@ -5579,19 +5585,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0D36391-A4E2-4B2A-AAD1-7B3B07126157}">
   <dimension ref="A2:I28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="29.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="29.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:9" ht="30.4" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="30.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="35" t="s">
         <v>78</v>
       </c>
@@ -5604,12 +5610,12 @@
       <c r="H2" s="35"/>
       <c r="I2" s="35"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="30" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="24" t="s">
         <v>80</v>
       </c>
@@ -5638,7 +5644,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="25" t="s">
         <v>89</v>
       </c>
@@ -5667,7 +5673,7 @@
         <v>1.0478950617283951</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="25" t="s">
         <v>90</v>
       </c>
@@ -5696,7 +5702,7 @@
         <v>0.66127963285024149</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="25" t="s">
         <v>91</v>
       </c>
@@ -5725,7 +5731,7 @@
         <v>0.42632098765432097</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="25" t="s">
         <v>92</v>
       </c>
@@ -5754,7 +5760,7 @@
         <v>0.29035215743440229</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="25" t="s">
         <v>93</v>
       </c>
@@ -5783,7 +5789,7 @@
         <v>0.43076923076923079</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="25" t="s">
         <v>94</v>
       </c>
@@ -5812,7 +5818,7 @@
         <v>0.76014999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="25" t="s">
         <v>95</v>
       </c>
@@ -5841,7 +5847,7 @@
         <v>0.9868055555555556</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="26" t="s">
         <v>96</v>
       </c>
@@ -5866,7 +5872,7 @@
       </c>
       <c r="I14" s="27"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C15" s="23">
         <v>0.62790697674418605</v>
       </c>
@@ -5880,12 +5886,12 @@
         <v>0.76663468337252794</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="30" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="24" t="s">
         <v>80</v>
       </c>
@@ -5914,7 +5920,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="25" t="s">
         <v>89</v>
       </c>
@@ -5943,7 +5949,7 @@
         <v>1.0104962025316455</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="25" t="s">
         <v>90</v>
       </c>
@@ -5972,7 +5978,7 @@
         <v>0.25263157894736843</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="25" t="s">
         <v>91</v>
       </c>
@@ -6001,7 +6007,7 @@
         <v>0.92666666666666664</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="25" t="s">
         <v>92</v>
       </c>
@@ -6030,7 +6036,7 @@
         <v>0.46149789029535865</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="25" t="s">
         <v>93</v>
       </c>
@@ -6059,7 +6065,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="25" t="s">
         <v>94</v>
       </c>
@@ -6088,7 +6094,7 @@
         <v>0.96381583333333343</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="25" t="s">
         <v>95</v>
       </c>
@@ -6117,7 +6123,7 @@
         <v>0.98919374999999987</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="26" t="s">
         <v>96</v>
       </c>
@@ -6142,7 +6148,7 @@
       </c>
       <c r="I27" s="27"/>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C28" s="23">
         <v>0.46</v>
       </c>
@@ -6168,43 +6174,43 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24D0948F-DE93-4FDE-A3AE-2B5CEA80AE20}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:AK295"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AK296"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="3" width="15.140625" customWidth="1"/>
+    <col min="2" max="3" width="15.109375" customWidth="1"/>
     <col min="4" max="5" width="25" customWidth="1"/>
-    <col min="6" max="6" width="24.5703125" customWidth="1"/>
-    <col min="8" max="8" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.28515625" customWidth="1"/>
-    <col min="10" max="10" width="31.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="11.5703125" customWidth="1"/>
-    <col min="13" max="13" width="10.28515625" customWidth="1"/>
+    <col min="6" max="6" width="24.5546875" customWidth="1"/>
+    <col min="8" max="8" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.33203125" customWidth="1"/>
+    <col min="10" max="10" width="31.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="11.5546875" customWidth="1"/>
+    <col min="13" max="13" width="10.33203125" customWidth="1"/>
     <col min="14" max="14" width="20" customWidth="1"/>
-    <col min="15" max="15" width="16.5703125" customWidth="1"/>
+    <col min="15" max="15" width="16.5546875" customWidth="1"/>
     <col min="16" max="16" width="10" customWidth="1"/>
     <col min="17" max="17" width="16" customWidth="1"/>
-    <col min="18" max="19" width="10.28515625" customWidth="1"/>
-    <col min="20" max="20" width="16.5703125" customWidth="1"/>
-    <col min="21" max="21" width="47.85546875" customWidth="1"/>
-    <col min="22" max="22" width="13.28515625" customWidth="1"/>
-    <col min="23" max="23" width="14.140625" customWidth="1"/>
-    <col min="24" max="24" width="16.5703125" customWidth="1"/>
-    <col min="25" max="25" width="47.85546875" customWidth="1"/>
-    <col min="26" max="26" width="17.85546875" customWidth="1"/>
+    <col min="18" max="19" width="10.33203125" customWidth="1"/>
+    <col min="20" max="20" width="16.5546875" customWidth="1"/>
+    <col min="21" max="21" width="47.88671875" customWidth="1"/>
+    <col min="22" max="22" width="13.33203125" customWidth="1"/>
+    <col min="23" max="23" width="14.109375" customWidth="1"/>
+    <col min="24" max="24" width="16.5546875" customWidth="1"/>
+    <col min="25" max="25" width="47.88671875" customWidth="1"/>
+    <col min="26" max="26" width="17.88671875" customWidth="1"/>
     <col min="27" max="27" width="25" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="16.5703125" customWidth="1"/>
-    <col min="32" max="32" width="47.85546875" customWidth="1"/>
-    <col min="33" max="33" width="17.85546875" customWidth="1"/>
-    <col min="34" max="34" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="16.5546875" customWidth="1"/>
+    <col min="32" max="32" width="47.88671875" customWidth="1"/>
+    <col min="33" max="33" width="17.88671875" customWidth="1"/>
+    <col min="34" max="34" width="23.109375" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="23.33203125" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="15" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="18.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A1" s="30" t="s">
         <v>1428</v>
       </c>
@@ -6317,7 +6323,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B2" s="6" t="s">
         <v>99</v>
       </c>
@@ -6415,7 +6421,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="3" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B3" s="6" t="s">
         <v>120</v>
       </c>
@@ -6500,7 +6506,7 @@
       </c>
       <c r="AG3" s="9"/>
     </row>
-    <row r="4" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B4" s="6" t="s">
         <v>128</v>
       </c>
@@ -6585,7 +6591,7 @@
       </c>
       <c r="AG4" s="9"/>
     </row>
-    <row r="5" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B5" s="6" t="s">
         <v>129</v>
       </c>
@@ -6670,7 +6676,7 @@
       </c>
       <c r="AG5" s="9"/>
     </row>
-    <row r="6" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B6" s="6" t="s">
         <v>1184</v>
       </c>
@@ -6741,7 +6747,7 @@
       </c>
       <c r="AG6" s="9"/>
     </row>
-    <row r="7" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
         <v>1193</v>
       </c>
@@ -6812,7 +6818,7 @@
       </c>
       <c r="AG7" s="9"/>
     </row>
-    <row r="8" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>1429</v>
       </c>
@@ -6903,7 +6909,7 @@
       </c>
       <c r="AG8" s="9"/>
     </row>
-    <row r="9" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>1429</v>
       </c>
@@ -6994,7 +7000,7 @@
       </c>
       <c r="AG9" s="9"/>
     </row>
-    <row r="10" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>1429</v>
       </c>
@@ -7085,7 +7091,7 @@
       </c>
       <c r="AG10" s="9"/>
     </row>
-    <row r="11" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>1429</v>
       </c>
@@ -7176,7 +7182,7 @@
       </c>
       <c r="AG11" s="9"/>
     </row>
-    <row r="12" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
         <v>1429</v>
       </c>
@@ -7280,7 +7286,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>1429</v>
       </c>
@@ -7368,7 +7374,7 @@
       </c>
       <c r="AG13" s="9"/>
     </row>
-    <row r="14" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>1430</v>
       </c>
@@ -7459,7 +7465,7 @@
       </c>
       <c r="AG14" s="9"/>
     </row>
-    <row r="15" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B15" s="6" t="s">
         <v>170</v>
       </c>
@@ -7547,7 +7553,7 @@
       </c>
       <c r="AG15" s="9"/>
     </row>
-    <row r="16" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B16" s="6" t="s">
         <v>182</v>
       </c>
@@ -7632,7 +7638,7 @@
       </c>
       <c r="AG16" s="9"/>
     </row>
-    <row r="17" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B17" s="6" t="s">
         <v>193</v>
       </c>
@@ -7717,7 +7723,7 @@
       </c>
       <c r="AG17" s="9"/>
     </row>
-    <row r="18" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B18" s="6" t="s">
         <v>298</v>
       </c>
@@ -7794,7 +7800,7 @@
       </c>
       <c r="AG18" s="9"/>
     </row>
-    <row r="19" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B19" s="6" t="s">
         <v>309</v>
       </c>
@@ -7873,7 +7879,7 @@
       </c>
       <c r="AG19" s="9"/>
     </row>
-    <row r="20" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B20" s="6" t="s">
         <v>320</v>
       </c>
@@ -7971,7 +7977,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="21" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B21" s="6" t="s">
         <v>327</v>
       </c>
@@ -8069,7 +8075,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="22" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B22" s="6" t="s">
         <v>328</v>
       </c>
@@ -8164,7 +8170,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="23" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B23" s="6" t="s">
         <v>329</v>
       </c>
@@ -8259,7 +8265,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="24" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B24" s="6" t="s">
         <v>330</v>
       </c>
@@ -8339,7 +8345,7 @@
       </c>
       <c r="AG24" s="9"/>
     </row>
-    <row r="25" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B25" s="6" t="s">
         <v>342</v>
       </c>
@@ -8424,7 +8430,7 @@
       </c>
       <c r="AG25" s="9"/>
     </row>
-    <row r="26" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B26" s="6" t="s">
         <v>349</v>
       </c>
@@ -8504,7 +8510,7 @@
       </c>
       <c r="AG26" s="9"/>
     </row>
-    <row r="27" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B27" s="6" t="s">
         <v>358</v>
       </c>
@@ -8584,7 +8590,7 @@
       </c>
       <c r="AG27" s="9"/>
     </row>
-    <row r="28" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B28" s="6" t="s">
         <v>359</v>
       </c>
@@ -8664,7 +8670,7 @@
       </c>
       <c r="AG28" s="9"/>
     </row>
-    <row r="29" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B29" s="6" t="s">
         <v>360</v>
       </c>
@@ -8765,7 +8771,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="30" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B30" s="6" t="s">
         <v>366</v>
       </c>
@@ -8866,7 +8872,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="31" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B31" s="6" t="s">
         <v>370</v>
       </c>
@@ -8964,7 +8970,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="32" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B32" s="6" t="s">
         <v>376</v>
       </c>
@@ -9057,7 +9063,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="33" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B33" s="6" t="s">
         <v>382</v>
       </c>
@@ -9140,7 +9146,7 @@
       </c>
       <c r="AG33" s="9"/>
     </row>
-    <row r="34" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B34" s="6" t="s">
         <v>388</v>
       </c>
@@ -9220,7 +9226,7 @@
       </c>
       <c r="AG34" s="9"/>
     </row>
-    <row r="35" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B35" s="6" t="s">
         <v>392</v>
       </c>
@@ -9305,7 +9311,7 @@
       </c>
       <c r="AG35" s="9"/>
     </row>
-    <row r="36" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B36" s="6" t="s">
         <v>396</v>
       </c>
@@ -9390,7 +9396,7 @@
       </c>
       <c r="AG36" s="9"/>
     </row>
-    <row r="37" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B37" s="6" t="s">
         <v>404</v>
       </c>
@@ -9475,7 +9481,7 @@
       </c>
       <c r="AG37" s="9"/>
     </row>
-    <row r="38" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B38" s="6" t="s">
         <v>405</v>
       </c>
@@ -9560,7 +9566,7 @@
       </c>
       <c r="AG38" s="9"/>
     </row>
-    <row r="39" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B39" s="6" t="s">
         <v>406</v>
       </c>
@@ -9645,7 +9651,7 @@
       </c>
       <c r="AG39" s="9"/>
     </row>
-    <row r="40" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B40" s="6" t="s">
         <v>407</v>
       </c>
@@ -9725,7 +9731,7 @@
       </c>
       <c r="AG40" s="9"/>
     </row>
-    <row r="41" spans="1:33" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:33" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A41" s="6" t="s">
         <v>1431</v>
       </c>
@@ -9813,7 +9819,7 @@
       </c>
       <c r="AG41" s="9"/>
     </row>
-    <row r="42" spans="1:33" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:33" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A42" s="6" t="s">
         <v>1431</v>
       </c>
@@ -9901,7 +9907,7 @@
       </c>
       <c r="AG42" s="9"/>
     </row>
-    <row r="43" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="6" t="s">
         <v>1431</v>
       </c>
@@ -9989,7 +9995,7 @@
       </c>
       <c r="AG43" s="9"/>
     </row>
-    <row r="44" spans="1:33" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:33" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A44" s="6" t="s">
         <v>1431</v>
       </c>
@@ -10077,7 +10083,7 @@
       </c>
       <c r="AG44" s="9"/>
     </row>
-    <row r="45" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B45" s="6" t="s">
         <v>423</v>
       </c>
@@ -10157,7 +10163,7 @@
       </c>
       <c r="AG45" s="9"/>
     </row>
-    <row r="46" spans="1:33" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:33" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A46" s="6" t="s">
         <v>1431</v>
       </c>
@@ -10236,7 +10242,7 @@
       </c>
       <c r="AG46" s="9"/>
     </row>
-    <row r="47" spans="1:33" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:33" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A47" s="6" t="s">
         <v>1431</v>
       </c>
@@ -10313,7 +10319,7 @@
       </c>
       <c r="AG47" s="9"/>
     </row>
-    <row r="48" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="6" t="s">
         <v>1431</v>
       </c>
@@ -10387,7 +10393,7 @@
       </c>
       <c r="AG48" s="9"/>
     </row>
-    <row r="49" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="6" t="s">
         <v>1431</v>
       </c>
@@ -10461,7 +10467,7 @@
       </c>
       <c r="AG49" s="9"/>
     </row>
-    <row r="50" spans="1:35" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:35" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A50" s="6" t="s">
         <v>1431</v>
       </c>
@@ -10540,7 +10546,7 @@
       </c>
       <c r="AG50" s="9"/>
     </row>
-    <row r="51" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B51" s="6" t="s">
         <v>439</v>
       </c>
@@ -10614,7 +10620,7 @@
       </c>
       <c r="AG51" s="9"/>
     </row>
-    <row r="52" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B52" s="6" t="s">
         <v>447</v>
       </c>
@@ -10697,7 +10703,7 @@
       </c>
       <c r="AG52" s="9"/>
     </row>
-    <row r="53" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B53" s="6" t="s">
         <v>453</v>
       </c>
@@ -10780,7 +10786,7 @@
       </c>
       <c r="AG53" s="9"/>
     </row>
-    <row r="54" spans="1:35" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:35" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A54" s="6" t="s">
         <v>1431</v>
       </c>
@@ -10871,7 +10877,7 @@
       </c>
       <c r="AG54" s="9"/>
     </row>
-    <row r="55" spans="1:35" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:35" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A55" s="6" t="s">
         <v>1431</v>
       </c>
@@ -10962,7 +10968,7 @@
       </c>
       <c r="AG55" s="9"/>
     </row>
-    <row r="56" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="6" t="s">
         <v>1431</v>
       </c>
@@ -11048,7 +11054,7 @@
       </c>
       <c r="AG56" s="9"/>
     </row>
-    <row r="57" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B57" s="6" t="s">
         <v>459</v>
       </c>
@@ -11133,7 +11139,7 @@
       </c>
       <c r="AG57" s="9"/>
     </row>
-    <row r="58" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B58" s="6" t="s">
         <v>464</v>
       </c>
@@ -11218,7 +11224,7 @@
       </c>
       <c r="AG58" s="9"/>
     </row>
-    <row r="59" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B59" s="6" t="s">
         <v>465</v>
       </c>
@@ -11303,7 +11309,7 @@
       </c>
       <c r="AG59" s="9"/>
     </row>
-    <row r="60" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B60" s="6" t="s">
         <v>466</v>
       </c>
@@ -11388,7 +11394,7 @@
       </c>
       <c r="AG60" s="9"/>
     </row>
-    <row r="61" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B61" s="6" t="s">
         <v>467</v>
       </c>
@@ -11489,7 +11495,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="62" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B62" s="6" t="s">
         <v>476</v>
       </c>
@@ -11585,7 +11591,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="63" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B63" s="6" t="s">
         <v>483</v>
       </c>
@@ -11681,7 +11687,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="64" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B64" s="6" t="s">
         <v>484</v>
       </c>
@@ -11777,7 +11783,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="65" spans="1:33" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:33" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A65" s="6" t="s">
         <v>1431</v>
       </c>
@@ -11865,7 +11871,7 @@
       </c>
       <c r="AG65" s="9"/>
     </row>
-    <row r="66" spans="1:33" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:33" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A66" s="6" t="s">
         <v>1431</v>
       </c>
@@ -11951,7 +11957,7 @@
       </c>
       <c r="AG66" s="9"/>
     </row>
-    <row r="67" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" s="6" t="s">
         <v>1431</v>
       </c>
@@ -12034,7 +12040,7 @@
       </c>
       <c r="AG67" s="9"/>
     </row>
-    <row r="68" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" s="6" t="s">
         <v>1431</v>
       </c>
@@ -12117,7 +12123,7 @@
       </c>
       <c r="AG68" s="9"/>
     </row>
-    <row r="69" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" s="6" t="s">
         <v>1431</v>
       </c>
@@ -12200,7 +12206,7 @@
       </c>
       <c r="AG69" s="9"/>
     </row>
-    <row r="70" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" s="6" t="s">
         <v>1431</v>
       </c>
@@ -12283,7 +12289,7 @@
       </c>
       <c r="AG70" s="9"/>
     </row>
-    <row r="71" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B71" s="6" t="s">
         <v>496</v>
       </c>
@@ -12368,7 +12374,7 @@
       </c>
       <c r="AG71" s="9"/>
     </row>
-    <row r="72" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B72" s="6" t="s">
         <v>501</v>
       </c>
@@ -12450,7 +12456,7 @@
       </c>
       <c r="AG72" s="9"/>
     </row>
-    <row r="73" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B73" s="6" t="s">
         <v>512</v>
       </c>
@@ -12532,7 +12538,7 @@
       </c>
       <c r="AG73" s="9"/>
     </row>
-    <row r="74" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B74" s="6" t="s">
         <v>513</v>
       </c>
@@ -12608,7 +12614,7 @@
       </c>
       <c r="AG74" s="9"/>
     </row>
-    <row r="75" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B75" s="6" t="s">
         <v>520</v>
       </c>
@@ -12688,7 +12694,7 @@
       </c>
       <c r="AG75" s="9"/>
     </row>
-    <row r="76" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B76" s="6" t="s">
         <v>527</v>
       </c>
@@ -12768,7 +12774,7 @@
       </c>
       <c r="AG76" s="9"/>
     </row>
-    <row r="77" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B77" s="6" t="s">
         <v>531</v>
       </c>
@@ -12848,7 +12854,7 @@
       </c>
       <c r="AG77" s="9"/>
     </row>
-    <row r="78" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B78" s="6" t="s">
         <v>535</v>
       </c>
@@ -12933,7 +12939,7 @@
       </c>
       <c r="AG78" s="9"/>
     </row>
-    <row r="79" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B79" s="6" t="s">
         <v>541</v>
       </c>
@@ -13010,7 +13016,7 @@
       </c>
       <c r="AG79" s="9"/>
     </row>
-    <row r="80" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B80" s="6" t="s">
         <v>551</v>
       </c>
@@ -13092,7 +13098,7 @@
       </c>
       <c r="AG80" s="9"/>
     </row>
-    <row r="81" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A81" s="6" t="s">
         <v>1432</v>
       </c>
@@ -13183,7 +13189,7 @@
       </c>
       <c r="AG81" s="9"/>
     </row>
-    <row r="82" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A82" s="6" t="s">
         <v>1432</v>
       </c>
@@ -13274,7 +13280,7 @@
       </c>
       <c r="AG82" s="9"/>
     </row>
-    <row r="83" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" s="6" t="s">
         <v>1432</v>
       </c>
@@ -13360,7 +13366,7 @@
       </c>
       <c r="AG83" s="9"/>
     </row>
-    <row r="84" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" s="6" t="s">
         <v>1432</v>
       </c>
@@ -13446,7 +13452,7 @@
       </c>
       <c r="AG84" s="9"/>
     </row>
-    <row r="85" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A85" s="6" t="s">
         <v>1434</v>
       </c>
@@ -13525,7 +13531,7 @@
       </c>
       <c r="AG85" s="9"/>
     </row>
-    <row r="86" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A86" s="6" t="s">
         <v>1435</v>
       </c>
@@ -13613,7 +13619,7 @@
       </c>
       <c r="AG86" s="9"/>
     </row>
-    <row r="87" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A87" s="6" t="s">
         <v>1435</v>
       </c>
@@ -13701,7 +13707,7 @@
       </c>
       <c r="AG87" s="9"/>
     </row>
-    <row r="88" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" s="6" t="s">
         <v>1435</v>
       </c>
@@ -13789,7 +13795,7 @@
       </c>
       <c r="AG88" s="9"/>
     </row>
-    <row r="89" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" s="6" t="s">
         <v>1435</v>
       </c>
@@ -13877,7 +13883,7 @@
       </c>
       <c r="AG89" s="9"/>
     </row>
-    <row r="90" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A90" s="6" t="s">
         <v>1435</v>
       </c>
@@ -13968,7 +13974,7 @@
       </c>
       <c r="AG90" s="9"/>
     </row>
-    <row r="91" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A91" s="6" t="s">
         <v>1433</v>
       </c>
@@ -14056,7 +14062,7 @@
       </c>
       <c r="AG91" s="9"/>
     </row>
-    <row r="92" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A92" s="6" t="s">
         <v>1433</v>
       </c>
@@ -14144,7 +14150,7 @@
       </c>
       <c r="AG92" s="9"/>
     </row>
-    <row r="93" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" s="6" t="s">
         <v>1433</v>
       </c>
@@ -14227,7 +14233,7 @@
       </c>
       <c r="AG93" s="9"/>
     </row>
-    <row r="94" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" s="6" t="s">
         <v>1433</v>
       </c>
@@ -14310,7 +14316,7 @@
       </c>
       <c r="AG94" s="9"/>
     </row>
-    <row r="95" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:37" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A95" s="6" t="s">
         <v>1432</v>
       </c>
@@ -14401,7 +14407,7 @@
       </c>
       <c r="AG95" s="9"/>
     </row>
-    <row r="96" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B96" s="6" t="s">
         <v>1195</v>
       </c>
@@ -14511,7 +14517,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="97" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B97" s="6" t="s">
         <v>1208</v>
       </c>
@@ -14590,7 +14596,7 @@
       </c>
       <c r="AG97" s="9"/>
     </row>
-    <row r="98" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B98" s="6" t="s">
         <v>1215</v>
       </c>
@@ -14669,7 +14675,7 @@
       </c>
       <c r="AG98" s="9"/>
     </row>
-    <row r="99" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B99" s="6" t="s">
         <v>1217</v>
       </c>
@@ -14754,7 +14760,7 @@
       </c>
       <c r="AG99" s="9"/>
     </row>
-    <row r="100" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B100" s="6" t="s">
         <v>605</v>
       </c>
@@ -14834,7 +14840,7 @@
       </c>
       <c r="AG100" s="9"/>
     </row>
-    <row r="101" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B101" s="6" t="s">
         <v>616</v>
       </c>
@@ -14917,7 +14923,7 @@
       </c>
       <c r="AG101" s="9"/>
     </row>
-    <row r="102" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B102" s="6" t="s">
         <v>622</v>
       </c>
@@ -14997,7 +15003,7 @@
       </c>
       <c r="AG102" s="9"/>
     </row>
-    <row r="103" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B103" s="6" t="s">
         <v>631</v>
       </c>
@@ -15077,7 +15083,7 @@
       </c>
       <c r="AG103" s="9"/>
     </row>
-    <row r="104" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B104" s="6" t="s">
         <v>642</v>
       </c>
@@ -15162,7 +15168,7 @@
       </c>
       <c r="AG104" s="9"/>
     </row>
-    <row r="105" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B105" s="6" t="s">
         <v>648</v>
       </c>
@@ -15247,7 +15253,7 @@
       </c>
       <c r="AG105" s="9"/>
     </row>
-    <row r="106" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B106" s="6" t="s">
         <v>649</v>
       </c>
@@ -15321,7 +15327,7 @@
       </c>
       <c r="AG106" s="9"/>
     </row>
-    <row r="107" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B107" s="6" t="s">
         <v>656</v>
       </c>
@@ -15395,7 +15401,7 @@
       </c>
       <c r="AG107" s="9"/>
     </row>
-    <row r="108" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B108" s="6" t="s">
         <v>1222</v>
       </c>
@@ -15474,7 +15480,7 @@
       </c>
       <c r="AG108" s="9"/>
     </row>
-    <row r="109" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B109" s="6" t="s">
         <v>1233</v>
       </c>
@@ -15553,7 +15559,7 @@
       </c>
       <c r="AG109" s="9"/>
     </row>
-    <row r="110" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B110" s="6" t="s">
         <v>1235</v>
       </c>
@@ -15632,7 +15638,7 @@
       </c>
       <c r="AG110" s="9"/>
     </row>
-    <row r="111" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B111" s="6" t="s">
         <v>1240</v>
       </c>
@@ -15711,7 +15717,7 @@
       </c>
       <c r="AG111" s="9"/>
     </row>
-    <row r="112" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B112" s="6" t="s">
         <v>1241</v>
       </c>
@@ -15790,7 +15796,7 @@
       </c>
       <c r="AG112" s="9"/>
     </row>
-    <row r="113" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B113" s="6" t="s">
         <v>1247</v>
       </c>
@@ -15875,7 +15881,7 @@
       </c>
       <c r="AG113" s="9"/>
     </row>
-    <row r="114" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B114" s="6" t="s">
         <v>1256</v>
       </c>
@@ -15951,7 +15957,7 @@
       </c>
       <c r="AG114" s="9"/>
     </row>
-    <row r="115" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B115" s="6" t="s">
         <v>1262</v>
       </c>
@@ -16027,7 +16033,7 @@
       </c>
       <c r="AG115" s="9"/>
     </row>
-    <row r="116" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B116" s="6" t="s">
         <v>1263</v>
       </c>
@@ -16106,7 +16112,7 @@
       </c>
       <c r="AG116" s="9"/>
     </row>
-    <row r="117" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B117" s="6" t="s">
         <v>1271</v>
       </c>
@@ -16185,7 +16191,7 @@
       </c>
       <c r="AG117" s="9"/>
     </row>
-    <row r="118" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B118" s="6" t="s">
         <v>1272</v>
       </c>
@@ -16270,7 +16276,7 @@
       </c>
       <c r="AG118" s="9"/>
     </row>
-    <row r="119" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B119" s="6" t="s">
         <v>1279</v>
       </c>
@@ -16349,7 +16355,7 @@
       </c>
       <c r="AG119" s="9"/>
     </row>
-    <row r="120" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B120" s="6" t="s">
         <v>1286</v>
       </c>
@@ -16428,7 +16434,7 @@
       </c>
       <c r="AG120" s="9"/>
     </row>
-    <row r="121" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B121" s="6" t="s">
         <v>1287</v>
       </c>
@@ -16507,7 +16513,7 @@
       </c>
       <c r="AG121" s="9"/>
     </row>
-    <row r="122" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B122" s="6" t="s">
         <v>1288</v>
       </c>
@@ -16592,7 +16598,7 @@
       </c>
       <c r="AG122" s="9"/>
     </row>
-    <row r="123" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B123" s="6" t="s">
         <v>1294</v>
       </c>
@@ -16674,7 +16680,7 @@
       </c>
       <c r="AG123" s="9"/>
     </row>
-    <row r="124" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B124" s="6" t="s">
         <v>1301</v>
       </c>
@@ -16756,7 +16762,7 @@
       </c>
       <c r="AG124" s="9"/>
     </row>
-    <row r="125" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B125" s="6" t="s">
         <v>1302</v>
       </c>
@@ -16838,7 +16844,7 @@
       </c>
       <c r="AG125" s="9"/>
     </row>
-    <row r="126" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B126" s="6" t="s">
         <v>1303</v>
       </c>
@@ -16920,7 +16926,7 @@
       </c>
       <c r="AG126" s="9"/>
     </row>
-    <row r="127" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B127" s="6" t="s">
         <v>1304</v>
       </c>
@@ -16996,7 +17002,7 @@
       </c>
       <c r="AG127" s="9"/>
     </row>
-    <row r="128" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B128" s="6" t="s">
         <v>1310</v>
       </c>
@@ -17067,7 +17073,7 @@
       </c>
       <c r="AG128" s="9"/>
     </row>
-    <row r="129" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B129" s="6" t="s">
         <v>1311</v>
       </c>
@@ -17147,7 +17153,7 @@
       </c>
       <c r="AG129" s="9"/>
     </row>
-    <row r="130" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B130" s="6" t="s">
         <v>1320</v>
       </c>
@@ -17227,7 +17233,7 @@
       </c>
       <c r="AG130" s="9"/>
     </row>
-    <row r="131" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B131" s="6" t="s">
         <v>1321</v>
       </c>
@@ -17307,7 +17313,7 @@
       </c>
       <c r="AG131" s="9"/>
     </row>
-    <row r="132" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B132" s="6" t="s">
         <v>1322</v>
       </c>
@@ -17383,7 +17389,7 @@
       </c>
       <c r="AG132" s="9"/>
     </row>
-    <row r="133" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B133" s="6" t="s">
         <v>1330</v>
       </c>
@@ -17459,7 +17465,7 @@
       </c>
       <c r="AG133" s="9"/>
     </row>
-    <row r="134" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B134" s="6" t="s">
         <v>1331</v>
       </c>
@@ -17535,7 +17541,7 @@
       </c>
       <c r="AG134" s="9"/>
     </row>
-    <row r="135" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B135" s="6" t="s">
         <v>1332</v>
       </c>
@@ -17609,7 +17615,7 @@
       </c>
       <c r="AG135" s="9"/>
     </row>
-    <row r="136" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B136" s="6" t="s">
         <v>1334</v>
       </c>
@@ -17683,7 +17689,7 @@
       </c>
       <c r="AG136" s="9"/>
     </row>
-    <row r="137" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B137" s="6" t="s">
         <v>1335</v>
       </c>
@@ -17762,7 +17768,7 @@
       </c>
       <c r="AG137" s="9"/>
     </row>
-    <row r="138" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B138" s="6" t="s">
         <v>1342</v>
       </c>
@@ -17841,7 +17847,7 @@
       </c>
       <c r="AG138" s="9"/>
     </row>
-    <row r="139" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B139" s="6" t="s">
         <v>1343</v>
       </c>
@@ -17920,7 +17926,7 @@
       </c>
       <c r="AG139" s="9"/>
     </row>
-    <row r="140" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B140" s="6" t="s">
         <v>1344</v>
       </c>
@@ -18005,7 +18011,7 @@
       </c>
       <c r="AG140" s="9"/>
     </row>
-    <row r="141" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B141" s="6" t="s">
         <v>1351</v>
       </c>
@@ -18079,7 +18085,7 @@
       </c>
       <c r="AG141" s="9"/>
     </row>
-    <row r="142" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B142" s="6" t="s">
         <v>1356</v>
       </c>
@@ -18150,7 +18156,7 @@
       </c>
       <c r="AG142" s="9"/>
     </row>
-    <row r="143" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B143" s="6" t="s">
         <v>1361</v>
       </c>
@@ -18232,7 +18238,7 @@
       </c>
       <c r="AG143" s="9"/>
     </row>
-    <row r="144" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B144" s="6" t="s">
         <v>1371</v>
       </c>
@@ -18311,7 +18317,7 @@
       </c>
       <c r="AG144" s="9"/>
     </row>
-    <row r="145" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B145" s="6" t="s">
         <v>664</v>
       </c>
@@ -18391,7 +18397,7 @@
       </c>
       <c r="AG145" s="9"/>
     </row>
-    <row r="146" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B146" s="6" t="s">
         <v>672</v>
       </c>
@@ -18473,7 +18479,7 @@
       </c>
       <c r="AG146" s="9"/>
     </row>
-    <row r="147" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B147" s="6" t="s">
         <v>680</v>
       </c>
@@ -18571,7 +18577,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="148" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B148" s="6" t="s">
         <v>689</v>
       </c>
@@ -18651,7 +18657,7 @@
       </c>
       <c r="AG148" s="9"/>
     </row>
-    <row r="149" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B149" s="6" t="s">
         <v>693</v>
       </c>
@@ -18731,7 +18737,7 @@
       </c>
       <c r="AG149" s="9"/>
     </row>
-    <row r="150" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B150" s="6" t="s">
         <v>698</v>
       </c>
@@ -18814,7 +18820,7 @@
       </c>
       <c r="AG150" s="9"/>
     </row>
-    <row r="151" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B151" s="6" t="s">
         <v>703</v>
       </c>
@@ -18896,7 +18902,7 @@
       </c>
       <c r="AG151" s="9"/>
     </row>
-    <row r="152" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B152" s="6" t="s">
         <v>711</v>
       </c>
@@ -18978,7 +18984,7 @@
       </c>
       <c r="AG152" s="9"/>
     </row>
-    <row r="153" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B153" s="6" t="s">
         <v>713</v>
       </c>
@@ -19079,7 +19085,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="154" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B154" s="6" t="s">
         <v>721</v>
       </c>
@@ -19180,7 +19186,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="155" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B155" s="6" t="s">
         <v>1378</v>
       </c>
@@ -19265,7 +19271,7 @@
       </c>
       <c r="AG155" s="9"/>
     </row>
-    <row r="156" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B156" s="6" t="s">
         <v>1390</v>
       </c>
@@ -19344,7 +19350,7 @@
       </c>
       <c r="AG156" s="9"/>
     </row>
-    <row r="157" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B157" s="6" t="s">
         <v>1398</v>
       </c>
@@ -19423,7 +19429,7 @@
       </c>
       <c r="AG157" s="9"/>
     </row>
-    <row r="158" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B158" s="6" t="s">
         <v>1404</v>
       </c>
@@ -19502,7 +19508,7 @@
       </c>
       <c r="AG158" s="9"/>
     </row>
-    <row r="159" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B159" s="6" t="s">
         <v>1405</v>
       </c>
@@ -19581,7 +19587,7 @@
       </c>
       <c r="AG159" s="9"/>
     </row>
-    <row r="160" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="2:35" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B160" s="6" t="s">
         <v>1411</v>
       </c>
@@ -19660,7 +19666,7 @@
       </c>
       <c r="AG160" s="9"/>
     </row>
-    <row r="161" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B161" s="6" t="s">
         <v>1417</v>
       </c>
@@ -19739,7 +19745,7 @@
       </c>
       <c r="AG161" s="9"/>
     </row>
-    <row r="162" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B162" s="6" t="s">
         <v>1424</v>
       </c>
@@ -19818,7 +19824,7 @@
       </c>
       <c r="AG162" s="9"/>
     </row>
-    <row r="163" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B163" s="6" t="s">
         <v>1425</v>
       </c>
@@ -19897,7 +19903,7 @@
       </c>
       <c r="AG163" s="9"/>
     </row>
-    <row r="164" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B164" s="6" t="s">
         <v>722</v>
       </c>
@@ -19982,7 +19988,7 @@
       </c>
       <c r="AG164" s="9"/>
     </row>
-    <row r="165" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B165" s="6" t="s">
         <v>730</v>
       </c>
@@ -20067,7 +20073,7 @@
       </c>
       <c r="AG165" s="9"/>
     </row>
-    <row r="166" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B166" s="6" t="s">
         <v>735</v>
       </c>
@@ -20177,7 +20183,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="167" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B167" s="6" t="s">
         <v>742</v>
       </c>
@@ -20248,7 +20254,7 @@
       </c>
       <c r="AG167" s="9"/>
     </row>
-    <row r="168" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B168" s="6" t="s">
         <v>748</v>
       </c>
@@ -20319,7 +20325,7 @@
       </c>
       <c r="AG168" s="9"/>
     </row>
-    <row r="169" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B169" s="6" t="s">
         <v>749</v>
       </c>
@@ -20407,7 +20413,7 @@
       </c>
       <c r="AG169" s="9"/>
     </row>
-    <row r="170" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B170" s="6" t="s">
         <v>756</v>
       </c>
@@ -20495,7 +20501,7 @@
       </c>
       <c r="AG170" s="9"/>
     </row>
-    <row r="171" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B171" s="6" t="s">
         <v>757</v>
       </c>
@@ -20578,7 +20584,7 @@
       </c>
       <c r="AG171" s="9"/>
     </row>
-    <row r="172" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B172" s="6" t="s">
         <v>758</v>
       </c>
@@ -20663,7 +20669,7 @@
       </c>
       <c r="AG172" s="9"/>
     </row>
-    <row r="173" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B173" s="6" t="s">
         <v>194</v>
       </c>
@@ -20748,7 +20754,7 @@
       </c>
       <c r="AG173" s="9"/>
     </row>
-    <row r="174" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B174" s="6" t="s">
         <v>209</v>
       </c>
@@ -20833,7 +20839,7 @@
       </c>
       <c r="AG174" s="9"/>
     </row>
-    <row r="175" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B175" s="6" t="s">
         <v>214</v>
       </c>
@@ -20918,7 +20924,7 @@
       </c>
       <c r="AG175" s="9"/>
     </row>
-    <row r="176" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B176" s="6" t="s">
         <v>223</v>
       </c>
@@ -21003,7 +21009,7 @@
       </c>
       <c r="AG176" s="9"/>
     </row>
-    <row r="177" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B177" s="6" t="s">
         <v>231</v>
       </c>
@@ -21088,7 +21094,7 @@
       </c>
       <c r="AG177" s="9"/>
     </row>
-    <row r="178" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B178" s="6" t="s">
         <v>237</v>
       </c>
@@ -21173,7 +21179,7 @@
       </c>
       <c r="AG178" s="9"/>
     </row>
-    <row r="179" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B179" s="6" t="s">
         <v>238</v>
       </c>
@@ -21258,7 +21264,7 @@
       </c>
       <c r="AG179" s="9"/>
     </row>
-    <row r="180" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B180" s="6" t="s">
         <v>243</v>
       </c>
@@ -21343,7 +21349,7 @@
       </c>
       <c r="AG180" s="9"/>
     </row>
-    <row r="181" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B181" s="6" t="s">
         <v>251</v>
       </c>
@@ -21428,7 +21434,7 @@
       </c>
       <c r="AG181" s="9"/>
     </row>
-    <row r="182" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B182" s="6" t="s">
         <v>253</v>
       </c>
@@ -21513,7 +21519,7 @@
       </c>
       <c r="AG182" s="9"/>
     </row>
-    <row r="183" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B183" s="6" t="s">
         <v>255</v>
       </c>
@@ -21598,7 +21604,7 @@
       </c>
       <c r="AG183" s="9"/>
     </row>
-    <row r="184" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B184" s="6" t="s">
         <v>257</v>
       </c>
@@ -21683,7 +21689,7 @@
       </c>
       <c r="AG184" s="9"/>
     </row>
-    <row r="185" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B185" s="6" t="s">
         <v>265</v>
       </c>
@@ -21763,7 +21769,7 @@
       </c>
       <c r="AG185" s="9"/>
     </row>
-    <row r="186" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B186" s="6" t="s">
         <v>267</v>
       </c>
@@ -21848,7 +21854,7 @@
       </c>
       <c r="AG186" s="9"/>
     </row>
-    <row r="187" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B187" s="6" t="s">
         <v>268</v>
       </c>
@@ -21933,7 +21939,7 @@
       </c>
       <c r="AG187" s="9"/>
     </row>
-    <row r="188" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B188" s="6" t="s">
         <v>269</v>
       </c>
@@ -22021,7 +22027,7 @@
       </c>
       <c r="AG188" s="9"/>
     </row>
-    <row r="189" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B189" s="6" t="s">
         <v>275</v>
       </c>
@@ -22106,7 +22112,7 @@
       </c>
       <c r="AG189" s="9"/>
     </row>
-    <row r="190" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B190" s="6" t="s">
         <v>283</v>
       </c>
@@ -22191,7 +22197,7 @@
       </c>
       <c r="AG190" s="9"/>
     </row>
-    <row r="191" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B191" s="6" t="s">
         <v>284</v>
       </c>
@@ -22276,7 +22282,7 @@
       </c>
       <c r="AG191" s="9"/>
     </row>
-    <row r="192" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B192" s="6" t="s">
         <v>285</v>
       </c>
@@ -22361,7 +22367,7 @@
       </c>
       <c r="AG192" s="9"/>
     </row>
-    <row r="193" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B193" s="6" t="s">
         <v>293</v>
       </c>
@@ -22446,7 +22452,7 @@
       </c>
       <c r="AG193" s="9"/>
     </row>
-    <row r="194" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B194" s="6" t="s">
         <v>294</v>
       </c>
@@ -22531,7 +22537,7 @@
       </c>
       <c r="AG194" s="9"/>
     </row>
-    <row r="195" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B195" s="6" t="s">
         <v>297</v>
       </c>
@@ -22616,7 +22622,7 @@
       </c>
       <c r="AG195" s="9"/>
     </row>
-    <row r="196" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="196" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B196" s="6" t="s">
         <v>764</v>
       </c>
@@ -22696,7 +22702,7 @@
       </c>
       <c r="AG196" s="9"/>
     </row>
-    <row r="197" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B197" s="6" t="s">
         <v>774</v>
       </c>
@@ -22770,7 +22776,7 @@
       </c>
       <c r="AG197" s="9"/>
     </row>
-    <row r="198" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B198" s="6" t="s">
         <v>782</v>
       </c>
@@ -22880,7 +22886,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="199" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B199" s="6" t="s">
         <v>787</v>
       </c>
@@ -22984,7 +22990,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="200" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B200" s="6" t="s">
         <v>790</v>
       </c>
@@ -23088,7 +23094,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="201" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B201" s="6" t="s">
         <v>791</v>
       </c>
@@ -23192,7 +23198,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="202" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B202" s="6" t="s">
         <v>792</v>
       </c>
@@ -23266,7 +23272,7 @@
       </c>
       <c r="AG202" s="9"/>
     </row>
-    <row r="203" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="203" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B203" s="6" t="s">
         <v>800</v>
       </c>
@@ -23351,7 +23357,7 @@
       </c>
       <c r="AG203" s="9"/>
     </row>
-    <row r="204" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="204" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B204" s="6" t="s">
         <v>805</v>
       </c>
@@ -23436,7 +23442,7 @@
       </c>
       <c r="AG204" s="9"/>
     </row>
-    <row r="205" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B205" s="6" t="s">
         <v>810</v>
       </c>
@@ -23521,7 +23527,7 @@
       </c>
       <c r="AG205" s="9"/>
     </row>
-    <row r="206" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="206" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B206" s="6" t="s">
         <v>815</v>
       </c>
@@ -23606,7 +23612,7 @@
       </c>
       <c r="AG206" s="9"/>
     </row>
-    <row r="207" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="207" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B207" s="6" t="s">
         <v>819</v>
       </c>
@@ -23691,7 +23697,7 @@
       </c>
       <c r="AG207" s="9"/>
     </row>
-    <row r="208" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B208" s="6" t="s">
         <v>824</v>
       </c>
@@ -23765,7 +23771,7 @@
       </c>
       <c r="AG208" s="9"/>
     </row>
-    <row r="209" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="209" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B209" s="6" t="s">
         <v>830</v>
       </c>
@@ -23839,7 +23845,7 @@
       </c>
       <c r="AG209" s="9"/>
     </row>
-    <row r="210" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B210" s="6" t="s">
         <v>831</v>
       </c>
@@ -23918,7 +23924,7 @@
       </c>
       <c r="AG210" s="9"/>
     </row>
-    <row r="211" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B211" s="6" t="s">
         <v>836</v>
       </c>
@@ -23992,7 +23998,7 @@
       </c>
       <c r="AG211" s="9"/>
     </row>
-    <row r="212" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B212" s="6" t="s">
         <v>839</v>
       </c>
@@ -24066,7 +24072,7 @@
       </c>
       <c r="AG212" s="9"/>
     </row>
-    <row r="213" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B213" s="6" t="s">
         <v>840</v>
       </c>
@@ -24151,7 +24157,7 @@
       </c>
       <c r="AG213" s="9"/>
     </row>
-    <row r="214" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B214" s="6" t="s">
         <v>849</v>
       </c>
@@ -24236,7 +24242,7 @@
       </c>
       <c r="AG214" s="9"/>
     </row>
-    <row r="215" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B215" s="6" t="s">
         <v>854</v>
       </c>
@@ -24316,7 +24322,7 @@
       </c>
       <c r="AG215" s="9"/>
     </row>
-    <row r="216" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B216" s="6" t="s">
         <v>859</v>
       </c>
@@ -24396,7 +24402,7 @@
       </c>
       <c r="AG216" s="9"/>
     </row>
-    <row r="217" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B217" s="6" t="s">
         <v>863</v>
       </c>
@@ -24476,7 +24482,7 @@
       </c>
       <c r="AG217" s="9"/>
     </row>
-    <row r="218" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B218" s="6" t="s">
         <v>867</v>
       </c>
@@ -24559,7 +24565,7 @@
       </c>
       <c r="AG218" s="9"/>
     </row>
-    <row r="219" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B219" s="6" t="s">
         <v>870</v>
       </c>
@@ -24639,7 +24645,7 @@
       </c>
       <c r="AG219" s="9"/>
     </row>
-    <row r="220" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B220" s="6" t="s">
         <v>877</v>
       </c>
@@ -24724,7 +24730,7 @@
       </c>
       <c r="AG220" s="9"/>
     </row>
-    <row r="221" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="221" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B221" s="6" t="s">
         <v>881</v>
       </c>
@@ -24804,7 +24810,7 @@
       </c>
       <c r="AG221" s="9"/>
     </row>
-    <row r="222" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="222" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B222" s="6" t="s">
         <v>882</v>
       </c>
@@ -24884,7 +24890,7 @@
       </c>
       <c r="AG222" s="9"/>
     </row>
-    <row r="223" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="223" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B223" s="6" t="s">
         <v>883</v>
       </c>
@@ -24964,7 +24970,7 @@
       </c>
       <c r="AG223" s="9"/>
     </row>
-    <row r="224" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="224" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B224" s="6" t="s">
         <v>884</v>
       </c>
@@ -25044,7 +25050,7 @@
       </c>
       <c r="AG224" s="9"/>
     </row>
-    <row r="225" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="225" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B225" s="6" t="s">
         <v>885</v>
       </c>
@@ -25129,7 +25135,7 @@
       </c>
       <c r="AG225" s="9"/>
     </row>
-    <row r="226" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="226" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B226" s="6" t="s">
         <v>889</v>
       </c>
@@ -25209,7 +25215,7 @@
       </c>
       <c r="AG226" s="9"/>
     </row>
-    <row r="227" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="227" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B227" s="6" t="s">
         <v>890</v>
       </c>
@@ -25289,7 +25295,7 @@
       </c>
       <c r="AG227" s="9"/>
     </row>
-    <row r="228" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="228" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B228" s="6" t="s">
         <v>891</v>
       </c>
@@ -25374,7 +25380,7 @@
       </c>
       <c r="AG228" s="9"/>
     </row>
-    <row r="229" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="229" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B229" s="6" t="s">
         <v>895</v>
       </c>
@@ -25454,7 +25460,7 @@
       </c>
       <c r="AG229" s="9"/>
     </row>
-    <row r="230" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="230" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B230" s="6" t="s">
         <v>904</v>
       </c>
@@ -25528,7 +25534,7 @@
       </c>
       <c r="AG230" s="9"/>
     </row>
-    <row r="231" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="231" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B231" s="6" t="s">
         <v>909</v>
       </c>
@@ -25616,7 +25622,7 @@
       </c>
       <c r="AG231" s="9"/>
     </row>
-    <row r="232" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="232" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B232" s="6" t="s">
         <v>919</v>
       </c>
@@ -25696,7 +25702,7 @@
       </c>
       <c r="AG232" s="9"/>
     </row>
-    <row r="233" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="233" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B233" s="6" t="s">
         <v>923</v>
       </c>
@@ -25776,7 +25782,7 @@
       </c>
       <c r="AG233" s="9"/>
     </row>
-    <row r="234" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="234" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B234" s="6" t="s">
         <v>927</v>
       </c>
@@ -25858,7 +25864,7 @@
       </c>
       <c r="AG234" s="9"/>
     </row>
-    <row r="235" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="235" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B235" s="6" t="s">
         <v>935</v>
       </c>
@@ -25940,7 +25946,7 @@
       </c>
       <c r="AG235" s="9"/>
     </row>
-    <row r="236" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="236" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B236" s="6" t="s">
         <v>936</v>
       </c>
@@ -26011,7 +26017,7 @@
       </c>
       <c r="AG236" s="9"/>
     </row>
-    <row r="237" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="237" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B237" s="6" t="s">
         <v>941</v>
       </c>
@@ -26082,7 +26088,7 @@
       </c>
       <c r="AG237" s="9"/>
     </row>
-    <row r="238" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="238" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B238" s="6" t="s">
         <v>942</v>
       </c>
@@ -26153,7 +26159,7 @@
       </c>
       <c r="AG238" s="9"/>
     </row>
-    <row r="239" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="239" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B239" s="6" t="s">
         <v>943</v>
       </c>
@@ -26227,7 +26233,7 @@
       </c>
       <c r="AG239" s="9"/>
     </row>
-    <row r="240" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="240" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B240" s="6" t="s">
         <v>949</v>
       </c>
@@ -26304,7 +26310,7 @@
       </c>
       <c r="AG240" s="9"/>
     </row>
-    <row r="241" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="241" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B241" s="6" t="s">
         <v>957</v>
       </c>
@@ -26381,7 +26387,7 @@
       </c>
       <c r="AG241" s="9"/>
     </row>
-    <row r="242" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="242" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B242" s="6" t="s">
         <v>962</v>
       </c>
@@ -26458,7 +26464,7 @@
       </c>
       <c r="AG242" s="9"/>
     </row>
-    <row r="243" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="243" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B243" s="6" t="s">
         <v>967</v>
       </c>
@@ -26535,7 +26541,7 @@
       </c>
       <c r="AG243" s="9"/>
     </row>
-    <row r="244" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B244" s="6" t="s">
         <v>972</v>
       </c>
@@ -26620,7 +26626,7 @@
       </c>
       <c r="AG244" s="9"/>
     </row>
-    <row r="245" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="245" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B245" s="6" t="s">
         <v>981</v>
       </c>
@@ -26705,7 +26711,7 @@
       </c>
       <c r="AG245" s="9"/>
     </row>
-    <row r="246" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B246" s="6" t="s">
         <v>986</v>
       </c>
@@ -26790,7 +26796,7 @@
       </c>
       <c r="AG246" s="9"/>
     </row>
-    <row r="247" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="247" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B247" s="6" t="s">
         <v>990</v>
       </c>
@@ -26873,7 +26879,7 @@
       </c>
       <c r="AG247" s="9"/>
     </row>
-    <row r="248" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="248" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B248" s="6" t="s">
         <v>995</v>
       </c>
@@ -26956,7 +26962,7 @@
       </c>
       <c r="AG248" s="9"/>
     </row>
-    <row r="249" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="249" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B249" s="6" t="s">
         <v>996</v>
       </c>
@@ -27039,7 +27045,7 @@
       </c>
       <c r="AG249" s="9"/>
     </row>
-    <row r="250" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="250" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B250" s="6" t="s">
         <v>1000</v>
       </c>
@@ -27122,7 +27128,7 @@
       </c>
       <c r="AG250" s="9"/>
     </row>
-    <row r="251" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="251" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B251" s="6" t="s">
         <v>1001</v>
       </c>
@@ -27202,7 +27208,7 @@
       </c>
       <c r="AG251" s="9"/>
     </row>
-    <row r="252" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="252" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B252" s="6" t="s">
         <v>1005</v>
       </c>
@@ -27282,7 +27288,7 @@
       </c>
       <c r="AG252" s="9"/>
     </row>
-    <row r="253" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="253" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B253" s="6" t="s">
         <v>1006</v>
       </c>
@@ -27362,7 +27368,7 @@
       </c>
       <c r="AG253" s="9"/>
     </row>
-    <row r="254" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="254" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B254" s="6" t="s">
         <v>1007</v>
       </c>
@@ -27442,7 +27448,7 @@
       </c>
       <c r="AG254" s="9"/>
     </row>
-    <row r="255" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="255" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B255" s="6" t="s">
         <v>1008</v>
       </c>
@@ -27522,7 +27528,7 @@
       </c>
       <c r="AG255" s="9"/>
     </row>
-    <row r="256" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="256" spans="2:33" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B256" s="6" t="s">
         <v>1009</v>
       </c>
@@ -27602,7 +27608,7 @@
       </c>
       <c r="AG256" s="9"/>
     </row>
-    <row r="257" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="257" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B257" s="6" t="s">
         <v>1010</v>
       </c>
@@ -27685,7 +27691,7 @@
       </c>
       <c r="AG257" s="9"/>
     </row>
-    <row r="258" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="258" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B258" s="6" t="s">
         <v>1014</v>
       </c>
@@ -27768,7 +27774,7 @@
       </c>
       <c r="AG258" s="9"/>
     </row>
-    <row r="259" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="259" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B259" s="6" t="s">
         <v>1015</v>
       </c>
@@ -27851,7 +27857,7 @@
       </c>
       <c r="AG259" s="9"/>
     </row>
-    <row r="260" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="260" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B260" s="6" t="s">
         <v>1019</v>
       </c>
@@ -27934,7 +27940,7 @@
       </c>
       <c r="AG260" s="9"/>
     </row>
-    <row r="261" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="261" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B261" s="6" t="s">
         <v>1020</v>
       </c>
@@ -28019,7 +28025,7 @@
       </c>
       <c r="AG261" s="9"/>
     </row>
-    <row r="262" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="262" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B262" s="6" t="s">
         <v>1024</v>
       </c>
@@ -28099,7 +28105,7 @@
       </c>
       <c r="AG262" s="9"/>
     </row>
-    <row r="263" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="263" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B263" s="6" t="s">
         <v>1031</v>
       </c>
@@ -28175,7 +28181,7 @@
       </c>
       <c r="AG263" s="9"/>
     </row>
-    <row r="264" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="264" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B264" s="6" t="s">
         <v>1036</v>
       </c>
@@ -28282,7 +28288,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="265" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="265" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B265" s="6" t="s">
         <v>1041</v>
       </c>
@@ -28367,7 +28373,7 @@
       </c>
       <c r="AG265" s="9"/>
     </row>
-    <row r="266" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="266" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B266" s="6" t="s">
         <v>1045</v>
       </c>
@@ -28452,7 +28458,7 @@
       </c>
       <c r="AG266" s="9"/>
     </row>
-    <row r="267" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="267" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B267" s="6" t="s">
         <v>1048</v>
       </c>
@@ -28537,7 +28543,7 @@
       </c>
       <c r="AG267" s="9"/>
     </row>
-    <row r="268" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="268" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B268" s="6" t="s">
         <v>1052</v>
       </c>
@@ -28622,7 +28628,7 @@
       </c>
       <c r="AG268" s="9"/>
     </row>
-    <row r="269" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="269" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B269" s="6" t="s">
         <v>1056</v>
       </c>
@@ -28729,7 +28735,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="270" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="270" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B270" s="6" t="s">
         <v>1067</v>
       </c>
@@ -28809,7 +28815,7 @@
       </c>
       <c r="AG270" s="9"/>
     </row>
-    <row r="271" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="271" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B271" s="6" t="s">
         <v>1074</v>
       </c>
@@ -28885,7 +28891,7 @@
       </c>
       <c r="AG271" s="9"/>
     </row>
-    <row r="272" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="272" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B272" s="6" t="s">
         <v>1080</v>
       </c>
@@ -28961,7 +28967,7 @@
       </c>
       <c r="AG272" s="9"/>
     </row>
-    <row r="273" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="273" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B273" s="6" t="s">
         <v>1081</v>
       </c>
@@ -29071,7 +29077,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="274" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="274" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B274" s="6" t="s">
         <v>1085</v>
       </c>
@@ -29142,7 +29148,7 @@
       </c>
       <c r="AG274" s="9"/>
     </row>
-    <row r="275" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="275" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B275" s="6" t="s">
         <v>1089</v>
       </c>
@@ -29237,7 +29243,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="276" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="276" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B276" s="6" t="s">
         <v>1095</v>
       </c>
@@ -29316,7 +29322,7 @@
       </c>
       <c r="AG276" s="9"/>
     </row>
-    <row r="277" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="277" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B277" s="6" t="s">
         <v>1101</v>
       </c>
@@ -29404,7 +29410,7 @@
       </c>
       <c r="AG277" s="9"/>
     </row>
-    <row r="278" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="278" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B278" s="6" t="s">
         <v>1105</v>
       </c>
@@ -29487,7 +29493,7 @@
       </c>
       <c r="AG278" s="9"/>
     </row>
-    <row r="279" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="279" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B279" s="6" t="s">
         <v>1106</v>
       </c>
@@ -29575,7 +29581,7 @@
       </c>
       <c r="AG279" s="9"/>
     </row>
-    <row r="280" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="280" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B280" s="6" t="s">
         <v>1107</v>
       </c>
@@ -29663,7 +29669,7 @@
       </c>
       <c r="AG280" s="9"/>
     </row>
-    <row r="281" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="281" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B281" s="6" t="s">
         <v>1108</v>
       </c>
@@ -29746,7 +29752,7 @@
       </c>
       <c r="AG281" s="9"/>
     </row>
-    <row r="282" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="282" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B282" s="6" t="s">
         <v>1109</v>
       </c>
@@ -29834,7 +29840,7 @@
       </c>
       <c r="AG282" s="9"/>
     </row>
-    <row r="283" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="283" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B283" s="6" t="s">
         <v>1112</v>
       </c>
@@ -29917,7 +29923,7 @@
       </c>
       <c r="AG283" s="9"/>
     </row>
-    <row r="284" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="284" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B284" s="6" t="s">
         <v>1113</v>
       </c>
@@ -30005,7 +30011,7 @@
       </c>
       <c r="AG284" s="9"/>
     </row>
-    <row r="285" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="285" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B285" s="6" t="s">
         <v>1114</v>
       </c>
@@ -30107,7 +30113,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="286" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="286" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B286" s="6" t="s">
         <v>1123</v>
       </c>
@@ -30187,7 +30193,7 @@
       </c>
       <c r="AG286" s="9"/>
     </row>
-    <row r="287" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="287" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B287" s="6" t="s">
         <v>1127</v>
       </c>
@@ -30272,7 +30278,7 @@
       </c>
       <c r="AG287" s="9"/>
     </row>
-    <row r="288" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="288" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B288" s="6" t="s">
         <v>1135</v>
       </c>
@@ -30352,7 +30358,7 @@
       </c>
       <c r="AG288" s="9"/>
     </row>
-    <row r="289" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B289" s="6" t="s">
         <v>1140</v>
       </c>
@@ -30462,7 +30468,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="290" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B290" s="6" t="s">
         <v>1144</v>
       </c>
@@ -30572,7 +30578,7 @@
         <v>1154</v>
       </c>
     </row>
-    <row r="291" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B291" s="6" t="s">
         <v>1155</v>
       </c>
@@ -30682,7 +30688,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="292" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B292" s="6" t="s">
         <v>1165</v>
       </c>
@@ -30792,7 +30798,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="293" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B293" s="6" t="s">
         <v>1171</v>
       </c>
@@ -30874,7 +30880,7 @@
       </c>
       <c r="AG293" s="9"/>
     </row>
-    <row r="294" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B294" s="6" t="s">
         <v>1176</v>
       </c>
@@ -30956,7 +30962,7 @@
       </c>
       <c r="AG294" s="9"/>
     </row>
-    <row r="295" spans="2:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:37" s="6" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B295" s="6" t="s">
         <v>1177</v>
       </c>
@@ -31035,6 +31041,62 @@
         <v>1154</v>
       </c>
       <c r="AG295" s="9"/>
+    </row>
+    <row r="296" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="A296" t="s">
+        <v>1433</v>
+      </c>
+      <c r="B296" t="s">
+        <v>1441</v>
+      </c>
+      <c r="C296" t="s">
+        <v>587</v>
+      </c>
+      <c r="D296" t="s">
+        <v>588</v>
+      </c>
+      <c r="E296" t="s">
+        <v>589</v>
+      </c>
+      <c r="F296" t="s">
+        <v>558</v>
+      </c>
+      <c r="G296" t="s">
+        <v>559</v>
+      </c>
+      <c r="H296">
+        <v>528</v>
+      </c>
+      <c r="I296" t="s">
+        <v>105</v>
+      </c>
+      <c r="J296" t="s">
+        <v>106</v>
+      </c>
+      <c r="K296">
+        <v>50.960856999999997</v>
+      </c>
+      <c r="L296">
+        <v>5.7935410000000003</v>
+      </c>
+      <c r="M296" t="s">
+        <v>107</v>
+      </c>
+      <c r="N296" t="s">
+        <v>108</v>
+      </c>
+      <c r="O296" t="s">
+        <v>94</v>
+      </c>
+      <c r="P296">
+        <v>550</v>
+      </c>
+      <c r="Q296" t="s">
+        <v>1442</v>
+      </c>
+      <c r="S296" t="s">
+        <v>110</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="B1:AK295" xr:uid="{4F45CA2E-3289-4008-8B81-764F641599B0}">
@@ -31072,6 +31134,16 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c95907cf-e9f9-4b92-a10f-5d23f887974d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100E03E5363D60F6E41BBDBD2986891499D" ma:contentTypeVersion="11" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="723753e909a658b81c41a8b79ae01792">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c95907cf-e9f9-4b92-a10f-5d23f887974d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e3777ca4d9a00e3a0fcbf4dc5e7e1334" ns2:_="">
     <xsd:import namespace="c95907cf-e9f9-4b92-a10f-5d23f887974d"/>
@@ -31255,16 +31327,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c95907cf-e9f9-4b92-a10f-5d23f887974d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -31275,24 +31337,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A82F1485-9B46-4DE7-8EF4-68C318268E4B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="c95907cf-e9f9-4b92-a10f-5d23f887974d"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55D8B328-D93F-4E0D-94E2-653BFEE7AE74}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
@@ -31311,6 +31355,24 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A82F1485-9B46-4DE7-8EF4-68C318268E4B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="c95907cf-e9f9-4b92-a10f-5d23f887974d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DF01CBF-A5C4-4282-859D-8EAB800F0387}">
   <ds:schemaRefs>

</xml_diff>